<commit_message>
Extend Sprint 1 timeline and move Airflow DAG to Sprint 2 (Decision 6)
</commit_message>
<xml_diff>
--- a/docs/gantt_chart.xlsx
+++ b/docs/gantt_chart.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ontario-wildfire-analytics\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ontario-wildfire-analytics\ontario-wildfire-impact-forecasting\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34DDBAAE-E6C3-452D-BF1F-959A4468EA92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E073B636-D1E5-4BE4-B09A-A96FAA66265A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Gantt Chart" sheetId="1" r:id="rId1"/>
@@ -365,8 +365,6 @@
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -382,6 +380,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -637,19 +637,19 @@
                   <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>14</c:v>
+                  <c:v>26</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>17</c:v>
+                  <c:v>35</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>23</c:v>
+                  <c:v>40</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>29</c:v>
+                  <c:v>45</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>33</c:v>
+                  <c:v>50</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -766,13 +766,13 @@
                   <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="2">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="3">
                   <c:v>10</c:v>
                 </c:pt>
-                <c:pt idx="3">
-                  <c:v>3</c:v>
-                </c:pt>
                 <c:pt idx="4">
-                  <c:v>6</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>6</c:v>
@@ -781,7 +781,7 @@
                   <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1189,249 +1189,249 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
     </row>
     <row r="4" spans="1:8" ht="39" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="3">
         <v>46220</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="3">
         <v>46223</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="2">
         <f t="shared" ref="E5:E12" si="0">NETWORKDAYS(C5,D5)</f>
         <v>2</v>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="2">
         <f t="shared" ref="F5:F12" si="1">NETWORKDAYS($C$5,C5)-1</f>
         <v>0</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="3">
         <v>46224</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="3">
         <v>46225</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="2">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="2">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="3">
         <v>46226</v>
       </c>
-      <c r="D7" s="5">
-        <v>46239</v>
-      </c>
-      <c r="E7" s="4">
+      <c r="D7" s="3">
+        <v>46255</v>
+      </c>
+      <c r="E7" s="2">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="F7" s="2">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C8" s="3">
+        <v>46258</v>
+      </c>
+      <c r="D8" s="3">
+        <v>46269</v>
+      </c>
+      <c r="E8" s="2">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="F7" s="4">
+      <c r="F8" s="2">
         <f t="shared" si="1"/>
+        <v>26</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" s="3">
+        <v>46270</v>
+      </c>
+      <c r="D9" s="3">
+        <v>46275</v>
+      </c>
+      <c r="E9" s="2">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="F9" s="2">
+        <f t="shared" si="1"/>
+        <v>35</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C8" s="5">
-        <v>46240</v>
-      </c>
-      <c r="D8" s="5">
-        <v>46244</v>
-      </c>
-      <c r="E8" s="4">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="F8" s="4">
-        <f t="shared" si="1"/>
-        <v>14</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C9" s="5">
-        <v>46245</v>
-      </c>
-      <c r="D9" s="5">
-        <v>46252</v>
-      </c>
-      <c r="E9" s="4">
+    <row r="10" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" s="3">
+        <v>46276</v>
+      </c>
+      <c r="D10" s="3">
+        <v>46283</v>
+      </c>
+      <c r="E10" s="2">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="F9" s="4">
+      <c r="F10" s="2">
         <f t="shared" si="1"/>
-        <v>17</v>
-      </c>
-      <c r="G9" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="C10" s="5">
-        <v>46253</v>
-      </c>
-      <c r="D10" s="5">
-        <v>46260</v>
-      </c>
-      <c r="E10" s="4">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="F10" s="4">
-        <f t="shared" si="1"/>
-        <v>23</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
     <row r="11" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C11" s="5">
-        <v>46261</v>
-      </c>
-      <c r="D11" s="5">
-        <v>46266</v>
-      </c>
-      <c r="E11" s="4">
+      <c r="C11" s="3">
+        <v>46284</v>
+      </c>
+      <c r="D11" s="3">
+        <v>46289</v>
+      </c>
+      <c r="E11" s="2">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="F11" s="4">
+      <c r="F11" s="2">
         <f t="shared" si="1"/>
-        <v>29</v>
-      </c>
-      <c r="G11" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C12" s="5">
-        <v>46267</v>
-      </c>
-      <c r="D12" s="5">
-        <v>46274</v>
-      </c>
-      <c r="E12" s="4">
+      <c r="C12" s="3">
+        <v>46290</v>
+      </c>
+      <c r="D12" s="3">
+        <v>46296</v>
+      </c>
+      <c r="E12" s="2">
         <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="F12" s="4">
+        <v>5</v>
+      </c>
+      <c r="F12" s="2">
         <f t="shared" si="1"/>
-        <v>33</v>
-      </c>
-      <c r="G12" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="G12" s="2" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1466,136 +1466,136 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
     </row>
     <row r="3" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="1" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="64.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="4" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="64.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="4" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="64.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="4" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="64.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="4" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="64.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="4" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="64.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="4" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="64.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="4" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="64.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="4" t="s">
         <v>77</v>
       </c>
     </row>
@@ -1618,65 +1618,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
     </row>
     <row r="3" spans="1:3" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="4" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="4" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="4" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="4" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="4" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="4" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="4" t="s">
         <v>54</v>
       </c>
     </row>

</xml_diff>